<commit_message>
chore(examples): refresh themed and dynamic example artifacts
</commit_message>
<xml_diff>
--- a/packages/examples/showcase/logical-vs-physical-summary/artifact/logical-vs-physical-summary.xlsx
+++ b/packages/examples/showcase/logical-vs-physical-summary/artifact/logical-vs-physical-summary.xlsx
@@ -8,7 +8,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+  <si>
+    <t>Logical Rows vs Physical Rows</t>
+  </si>
   <si>
     <t>Customer</t>
   </si>
@@ -167,7 +170,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -181,111 +184,107 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3">
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="3">
         <v>10</v>
       </c>
-      <c r="D2" s="3">
-        <f>ROUND(AVERAGE(C2:C4),2)</f>
-      </c>
-      <c r="E2" s="3">
-        <f>ROUND(SUM(C2:C4),2)</f>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="3">
-        <v>20</v>
-      </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
+      <c r="D3" s="3">
+        <f>ROUND(AVERAGE(C3:C5),2)</f>
+      </c>
+      <c r="E3" s="3">
+        <f>ROUND(SUM(C3:C5),2)</f>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="3">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="3">
+        <v>30</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="3">
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="3">
         <v>100</v>
       </c>
-      <c r="D5" s="3">
-        <f>ROUND(AVERAGE(C5:C6),2)</f>
-      </c>
-      <c r="E5" s="3">
-        <f>ROUND(SUM(C5:C6),2)</f>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="3">
+      <c r="D6" s="3">
+        <f>ROUND(AVERAGE(C6:C7),2)</f>
+      </c>
+      <c r="E6" s="3">
+        <f>ROUND(SUM(C6:C7),2)</f>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="3">
         <v>200</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="2" t="s">
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="3">
+      <c r="C8" s="3">
         <v>80</v>
       </c>
-      <c r="D7" s="3">
-        <f>ROUND(AVERAGE(C7:C10),2)</f>
-      </c>
-      <c r="E7" s="3">
-        <f>ROUND(SUM(C7:C10),2)</f>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="3">
-        <v>120</v>
-      </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
+      <c r="D8" s="3">
+        <f>ROUND(AVERAGE(C8:C11),2)</f>
+      </c>
+      <c r="E8" s="3">
+        <f>ROUND(SUM(C8:C11),2)</f>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="3">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -294,27 +293,26 @@
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="3">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="5">
-        <f>SUM(C2:C10)</f>
-      </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="3">
+        <v>160</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="5">
-        <f>AVERAGE(C2:C10)</f>
+        <f>SUM(C3:C11)</f>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
@@ -324,11 +322,9 @@
         <v>12</v>
       </c>
       <c r="C13" s="5">
-        <f>AVERAGE(AVERAGE(C2:C4),AVERAGE(C5:C6),AVERAGE(C7:C10))</f>
-      </c>
-      <c r="D13" s="5">
-        <f>AVERAGE(AVERAGE(D2:D4),AVERAGE(D5:D6),AVERAGE(D7:D10))</f>
-      </c>
+        <f>AVERAGE(C3:C11)</f>
+      </c>
+      <c r="D13" s="4"/>
       <c r="E13" s="4"/>
     </row>
     <row r="14" ht="30" customHeight="1">
@@ -336,27 +332,40 @@
         <v>13</v>
       </c>
       <c r="C14" s="5">
-        <f>SUM(AVERAGE(C2:C4),AVERAGE(C5:C6),AVERAGE(C7:C10))</f>
-      </c>
-      <c r="D14" s="4"/>
-      <c r="E14" s="5">
-        <f>SUM(AVERAGE(E2:E4),AVERAGE(E5:E6),AVERAGE(E7:E10))</f>
+        <f>AVERAGE(AVERAGE(C3:C5),AVERAGE(C6:C7),AVERAGE(C8:C11))</f>
+      </c>
+      <c r="D14" s="5">
+        <f>AVERAGE(AVERAGE(D3:D5),AVERAGE(D6:D7),AVERAGE(D8:D11))</f>
+      </c>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="5">
+        <f>SUM(AVERAGE(C3:C5),AVERAGE(C6:C7),AVERAGE(C8:C11))</f>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="5">
+        <f>SUM(AVERAGE(E3:E5),AVERAGE(E6:E7),AVERAGE(E8:E11))</f>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="D2:D4"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="D7:D10"/>
-    <mergeCell ref="E7:E10"/>
+  <mergeCells count="13">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="D8:D11"/>
+    <mergeCell ref="E8:E11"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>